<commit_message>
A bunch of elemental changes
</commit_message>
<xml_diff>
--- a/public/effects.xlsx
+++ b/public/effects.xlsx
@@ -1013,7 +1013,7 @@
         <v>1</v>
       </c>
       <c r="G25" t="str">
-        <v>Value</v>
+        <v>Number</v>
       </c>
     </row>
     <row r="26">
@@ -1040,13 +1040,49 @@
       </c>
     </row>
     <row r="27">
+      <c r="A27" t="str">
+        <v>boosted</v>
+      </c>
       <c r="B27" t="str">
-        <v>_x000d_</v>
+        <v>Passive</v>
+      </c>
+      <c r="C27" t="str">
+        <v>+</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Increases energy at turn start</v>
+      </c>
+      <c r="E27" t="str">
+        <v>+X energy at turn start</v>
+      </c>
+      <c r="F27" t="str">
+        <v>1</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Number</v>
       </c>
     </row>
     <row r="28">
+      <c r="A28" t="str">
+        <v>healthy</v>
+      </c>
       <c r="B28" t="str">
-        <v>_x000d_</v>
+        <v>Passive</v>
+      </c>
+      <c r="C28" t="str">
+        <v>+</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Increases Max HP</v>
+      </c>
+      <c r="E28" t="str">
+        <v>+X Max HP</v>
+      </c>
+      <c r="F28" t="str">
+        <v>10</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Number</v>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
Add brittle as effect
</commit_message>
<xml_diff>
--- a/public/effects.xlsx
+++ b/public/effects.xlsx
@@ -1086,8 +1086,26 @@
       </c>
     </row>
     <row r="29">
+      <c r="A29" t="str">
+        <v>brittle</v>
+      </c>
       <c r="B29" t="str">
-        <v>_x000d_</v>
+        <v>Element</v>
+      </c>
+      <c r="C29" t="str">
+        <v>+</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Consumed after X uses in a FORMULA</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Consumed after X uses in a FORMULA</v>
+      </c>
+      <c r="F29" t="str">
+        <v>1</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Number</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
Move level >> Rank. Add starting effects for all elements
</commit_message>
<xml_diff>
--- a/public/effects.xlsx
+++ b/public/effects.xlsx
@@ -397,18 +397,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:J34"/>
   <cols>
-    <col min="1" max="1" width="29.50390625" customWidth="1"/>
-    <col min="2" max="2" width="29.50390625" customWidth="1"/>
-    <col min="3" max="3" width="29.50390625" customWidth="1"/>
-    <col min="4" max="4" width="46.6640625" customWidth="1"/>
-    <col min="5" max="5" width="60.00390625" customWidth="1"/>
-    <col min="6" max="6" width="29.50390625" customWidth="1"/>
-    <col min="7" max="7" width="29.50390625" customWidth="1"/>
-    <col min="8" max="8" width="29.50390625" customWidth="1"/>
-    <col min="9" max="9" width="29.50390625" customWidth="1"/>
-    <col min="10" max="10" width="16.6640625" customWidth="1"/>
+    <col min="1" max="1" width="42.00390625" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" customWidth="1"/>
+    <col min="3" max="3" width="42.00390625" customWidth="1"/>
+    <col min="4" max="4" width="42.00390625" customWidth="1"/>
+    <col min="5" max="5" width="50.00390625" customWidth="1"/>
+    <col min="6" max="6" width="50.00390625" customWidth="1"/>
+    <col min="7" max="7" width="42.00390625" customWidth="1"/>
+    <col min="8" max="8" width="42.00390625" customWidth="1"/>
+    <col min="9" max="9" width="42.00390625" customWidth="1"/>
+    <col min="10" max="10" width="42.00390625" customWidth="1"/>
     <col min="11" max="11" width="16.6640625" customWidth="1"/>
     <col min="12" max="12" width="16.6640625" customWidth="1"/>
     <col min="13" max="13" width="16.6640625" customWidth="1"/>
@@ -432,27 +432,30 @@
         <v>Effect</v>
       </c>
       <c r="B1" t="str">
+        <v>Type</v>
+      </c>
+      <c r="C1" t="str">
         <v>Effect Type</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Growth</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Short Description</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Long Description</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Amount</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Amount Type</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Duration</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Target</v>
       </c>
     </row>
@@ -461,24 +464,27 @@
         <v>consume</v>
       </c>
       <c r="B2" t="str">
-        <v>Active</v>
+        <v>Fire</v>
       </c>
       <c r="C2" t="str">
+        <v>Active</v>
+      </c>
+      <c r="D2" t="str">
         <v>-</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>When used, reduce your Max HP by X</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>Each time this attack is used, reduces attackers max HP by X.</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>5</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>Number</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>self</v>
       </c>
     </row>
@@ -487,21 +493,24 @@
         <v>hardened</v>
       </c>
       <c r="B3" t="str">
-        <v>Active</v>
+        <v>Earth</v>
       </c>
       <c r="C3" t="str">
-        <v>+</v>
+        <v>Active</v>
       </c>
       <c r="D3" t="str">
+        <v>+</v>
+      </c>
+      <c r="E3" t="str">
         <v>Increase damage based on shield</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>Gets +X% attack power per shield that the entity has</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>5</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>Percent</v>
       </c>
     </row>
@@ -510,24 +519,27 @@
         <v>soaker</v>
       </c>
       <c r="B4" t="str">
+        <v>Water</v>
+      </c>
+      <c r="C4" t="str">
         <v>Stack</v>
       </c>
-      <c r="C4" t="str">
-        <v>+</v>
-      </c>
       <c r="D4" t="str">
+        <v>+</v>
+      </c>
+      <c r="E4" t="str">
         <v>Applies SOAK stacks</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>Applies X SOAK stack(s) on hit</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>1</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>Number</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>3</v>
       </c>
     </row>
@@ -536,22 +548,25 @@
         <v>follow up</v>
       </c>
       <c r="B5" t="str">
-        <v>Active</v>
+        <v>Air</v>
       </c>
       <c r="C5" t="str">
-        <v>+</v>
+        <v>Active</v>
       </c>
       <c r="D5" t="str">
+        <v>+</v>
+      </c>
+      <c r="E5" t="str">
         <v>Increase power when used consecutively</v>
       </c>
-      <c r="E5" t="str" xml:space="preserve">
+      <c r="F5" t="str" xml:space="preserve">
         <v xml:space="preserve">If your next attack is this attack, it deals X% additional damage. 
 Can stack, but does not carry over across turns</v>
       </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
         <v>50</v>
       </c>
-      <c r="G5" t="str">
+      <c r="H5" t="str">
         <v>Percent</v>
       </c>
     </row>
@@ -560,24 +575,27 @@
         <v>burn</v>
       </c>
       <c r="B6" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="C6" t="str">
         <v>Stack</v>
       </c>
-      <c r="C6" t="str">
-        <v>+</v>
-      </c>
       <c r="D6" t="str">
+        <v>+</v>
+      </c>
+      <c r="E6" t="str">
         <v>Applies BURN stacks</v>
       </c>
-      <c r="E6" t="str">
+      <c r="F6" t="str">
         <v>Applies X BURN stack(s) on hit</v>
       </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
         <v>1</v>
       </c>
-      <c r="G6" t="str">
+      <c r="H6" t="str">
         <v>Number</v>
       </c>
-      <c r="H6" t="str">
+      <c r="I6" t="str">
         <v>3</v>
       </c>
     </row>
@@ -586,27 +604,30 @@
         <v>thorns</v>
       </c>
       <c r="B7" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="C7" t="str">
         <v>Stack</v>
       </c>
-      <c r="C7" t="str">
-        <v>+</v>
-      </c>
       <c r="D7" t="str">
+        <v>+</v>
+      </c>
+      <c r="E7" t="str">
         <v>Applies THORN stacks to self</v>
       </c>
-      <c r="E7" t="str">
+      <c r="F7" t="str">
         <v>Applies X THORNS stack(s) on self when used</v>
       </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
         <v>1</v>
       </c>
-      <c r="G7" t="str">
+      <c r="H7" t="str">
         <v>Number</v>
       </c>
-      <c r="H7" t="str">
+      <c r="I7" t="str">
         <v>2</v>
       </c>
-      <c r="I7" t="str">
+      <c r="J7" t="str">
         <v>self</v>
       </c>
     </row>
@@ -615,21 +636,24 @@
         <v xml:space="preserve">power combo </v>
       </c>
       <c r="B8" t="str">
-        <v>Active</v>
+        <v>Water</v>
       </c>
       <c r="C8" t="str">
-        <v>+</v>
+        <v>Active</v>
       </c>
       <c r="D8" t="str">
+        <v>+</v>
+      </c>
+      <c r="E8" t="str">
         <v>If next attack is ELEMENT, it deals more damage</v>
       </c>
-      <c r="E8" t="str">
+      <c r="F8" t="str">
         <v>Your next attack deals +X% more damage if it is the associated type</v>
       </c>
-      <c r="F8" t="str">
+      <c r="G8" t="str">
         <v>50</v>
       </c>
-      <c r="G8" t="str">
+      <c r="H8" t="str">
         <v>Percent</v>
       </c>
     </row>
@@ -638,23 +662,26 @@
         <v>float</v>
       </c>
       <c r="B9" t="str">
+        <v>Air</v>
+      </c>
+      <c r="C9" t="str">
         <v>Passive</v>
       </c>
-      <c r="C9" t="str">
-        <v>+</v>
-      </c>
-      <c r="D9" t="str" xml:space="preserve">
+      <c r="D9" t="str">
+        <v>+</v>
+      </c>
+      <c r="E9" t="str" xml:space="preserve">
         <v xml:space="preserve">Increase LIGHTNING Damage
 Decrease EARTH damage</v>
       </c>
-      <c r="E9" t="str" xml:space="preserve">
+      <c r="F9" t="str" xml:space="preserve">
         <v xml:space="preserve">Reduce EARTH damage taken by X%
 Increase LIGHTNING damage taken by X%</v>
       </c>
-      <c r="F9" t="str">
+      <c r="G9" t="str">
         <v>50</v>
       </c>
-      <c r="G9" t="str">
+      <c r="H9" t="str">
         <v>Percent</v>
       </c>
     </row>
@@ -663,21 +690,24 @@
         <v>rage</v>
       </c>
       <c r="B10" t="str">
-        <v>Active</v>
+        <v>Fire</v>
       </c>
       <c r="C10" t="str">
-        <v>+</v>
+        <v>Active</v>
       </c>
       <c r="D10" t="str">
+        <v>+</v>
+      </c>
+      <c r="E10" t="str">
         <v>The lower your health, the higher the damage</v>
       </c>
-      <c r="E10" t="str">
+      <c r="F10" t="str">
         <v>Increase damage by X for every 1 health missing</v>
       </c>
-      <c r="F10" t="str">
+      <c r="G10" t="str">
         <v>1</v>
       </c>
-      <c r="G10" t="str">
+      <c r="H10" t="str">
         <v>Number</v>
       </c>
     </row>
@@ -686,27 +716,30 @@
         <v>energize</v>
       </c>
       <c r="B11" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="C11" t="str">
         <v>Stack</v>
       </c>
-      <c r="C11" t="str">
+      <c r="D11" t="str">
         <v>=</v>
       </c>
-      <c r="D11" t="str">
+      <c r="E11" t="str">
         <v>Start you next turn with more energy</v>
       </c>
-      <c r="E11" t="str">
+      <c r="F11" t="str">
         <v>Each stack provides +X energy at the start of your next turn!</v>
       </c>
-      <c r="F11" t="str">
+      <c r="G11" t="str">
         <v>1</v>
       </c>
-      <c r="G11" t="str">
+      <c r="H11" t="str">
         <v>Number</v>
       </c>
-      <c r="H11" t="str">
+      <c r="I11" t="str">
         <v>2</v>
       </c>
-      <c r="I11" t="str">
+      <c r="J11" t="str">
         <v>self</v>
       </c>
     </row>
@@ -715,21 +748,24 @@
         <v>heal</v>
       </c>
       <c r="B12" t="str">
-        <v>Active</v>
+        <v>Water</v>
       </c>
       <c r="C12" t="str">
-        <v>+</v>
+        <v>Active</v>
       </c>
       <c r="D12" t="str">
+        <v>+</v>
+      </c>
+      <c r="E12" t="str">
         <v>Restores HP</v>
       </c>
-      <c r="E12" t="str">
+      <c r="F12" t="str">
         <v>Restores X HP</v>
       </c>
-      <c r="F12" t="str">
+      <c r="G12" t="str">
         <v>5</v>
       </c>
-      <c r="G12" t="str">
+      <c r="H12" t="str">
         <v>Number</v>
       </c>
     </row>
@@ -738,21 +774,24 @@
         <v>energy combo</v>
       </c>
       <c r="B13" t="str">
-        <v>Active</v>
+        <v>Air</v>
       </c>
       <c r="C13" t="str">
-        <v>+</v>
+        <v>Active</v>
       </c>
       <c r="D13" t="str">
+        <v>+</v>
+      </c>
+      <c r="E13" t="str">
         <v>If next attack is the same element, it costs less energy</v>
       </c>
-      <c r="E13" t="str">
+      <c r="F13" t="str">
         <v>Next attack costs X less energy if it is the associated type</v>
       </c>
-      <c r="F13" t="str">
+      <c r="G13" t="str">
         <v>1</v>
       </c>
-      <c r="G13" t="str">
+      <c r="H13" t="str">
         <v>Number</v>
       </c>
     </row>
@@ -761,24 +800,27 @@
         <v>combust</v>
       </c>
       <c r="B14" t="str">
-        <v>Active</v>
+        <v>Fire</v>
       </c>
       <c r="C14" t="str">
+        <v>Active</v>
+      </c>
+      <c r="D14" t="str">
         <v>-</v>
       </c>
-      <c r="D14" t="str">
+      <c r="E14" t="str">
         <v>On use, deal damage to self</v>
       </c>
-      <c r="E14" t="str">
+      <c r="F14" t="str">
         <v>When attacking, deals X% of the damage to yourself</v>
       </c>
-      <c r="F14" t="str">
+      <c r="G14" t="str">
         <v>10</v>
       </c>
-      <c r="G14" t="str">
-        <v>Percent</v>
-      </c>
-      <c r="I14" t="str">
+      <c r="H14" t="str">
+        <v>Percent</v>
+      </c>
+      <c r="J14" t="str">
         <v>self</v>
       </c>
     </row>
@@ -787,21 +829,24 @@
         <v>charge</v>
       </c>
       <c r="B15" t="str">
-        <v>Active</v>
+        <v>Earth</v>
       </c>
       <c r="C15" t="str">
-        <v>+</v>
+        <v>Active</v>
       </c>
       <c r="D15" t="str">
+        <v>+</v>
+      </c>
+      <c r="E15" t="str">
         <v>Increase damage based on energy cost</v>
       </c>
-      <c r="E15" t="str">
+      <c r="F15" t="str">
         <v>Deals +X% more damage for each energy in its cost</v>
       </c>
-      <c r="F15" t="str">
+      <c r="G15" t="str">
         <v>50</v>
       </c>
-      <c r="G15" t="str">
+      <c r="H15" t="str">
         <v>Percent</v>
       </c>
     </row>
@@ -810,21 +855,24 @@
         <v>shield</v>
       </c>
       <c r="B16" t="str">
-        <v>Active</v>
+        <v>Water, Earth</v>
       </c>
       <c r="C16" t="str">
+        <v>Active</v>
+      </c>
+      <c r="D16" t="str">
         <v>=</v>
       </c>
-      <c r="D16" t="str">
+      <c r="E16" t="str">
         <v>Absorbs incoming damage</v>
       </c>
-      <c r="E16" t="str">
+      <c r="F16" t="str">
         <v>Absorbs X damage per 1 shield</v>
       </c>
-      <c r="F16" t="str">
+      <c r="G16" t="str">
         <v>1</v>
       </c>
-      <c r="G16" t="str">
+      <c r="H16" t="str">
         <v>Number</v>
       </c>
     </row>
@@ -833,24 +881,27 @@
         <v>freeze</v>
       </c>
       <c r="B17" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="C17" t="str">
         <v>Stack</v>
       </c>
-      <c r="C17" t="str">
+      <c r="D17" t="str">
         <v>=</v>
       </c>
-      <c r="D17" t="str">
+      <c r="E17" t="str">
         <v>Transform SOAK stacks into ICE stacks</v>
       </c>
-      <c r="E17" t="str">
+      <c r="F17" t="str">
         <v>Transforms X% of SOAK stacks into ICE stacks</v>
       </c>
-      <c r="F17" t="str">
+      <c r="G17" t="str">
         <v>100</v>
       </c>
-      <c r="G17" t="str">
-        <v>Percent</v>
-      </c>
       <c r="H17" t="str">
+        <v>Percent</v>
+      </c>
+      <c r="I17" t="str">
         <v>1</v>
       </c>
     </row>
@@ -859,21 +910,24 @@
         <v>exponential</v>
       </c>
       <c r="B18" t="str">
-        <v>Active</v>
+        <v>Fire, Earth</v>
       </c>
       <c r="C18" t="str">
-        <v>+</v>
+        <v>Active</v>
       </c>
       <c r="D18" t="str">
+        <v>+</v>
+      </c>
+      <c r="E18" t="str">
         <v>Permanently increase damage on use</v>
       </c>
-      <c r="E18" t="str">
+      <c r="F18" t="str">
         <v>Each time this attack is used, permanently increase its damage by X%</v>
       </c>
-      <c r="F18" t="str">
+      <c r="G18" t="str">
         <v>10</v>
       </c>
-      <c r="G18" t="str">
+      <c r="H18" t="str">
         <v>Percent</v>
       </c>
     </row>
@@ -882,21 +936,24 @@
         <v>resistant</v>
       </c>
       <c r="B19" t="str">
+        <v>-</v>
+      </c>
+      <c r="C19" t="str">
         <v>Passive</v>
       </c>
-      <c r="C19" t="str">
-        <v>+</v>
-      </c>
       <c r="D19" t="str">
+        <v>+</v>
+      </c>
+      <c r="E19" t="str">
         <v>Reduce ELEMENT damage</v>
       </c>
-      <c r="E19" t="str">
+      <c r="F19" t="str">
         <v>Reduce ELEMENT damage received by X%</v>
       </c>
-      <c r="F19" t="str">
+      <c r="G19" t="str">
         <v>10</v>
       </c>
-      <c r="G19" t="str">
+      <c r="H19" t="str">
         <v>Percent</v>
       </c>
     </row>
@@ -905,21 +962,24 @@
         <v>vulnerable</v>
       </c>
       <c r="B20" t="str">
+        <v>-</v>
+      </c>
+      <c r="C20" t="str">
         <v>Passive</v>
       </c>
-      <c r="C20" t="str">
+      <c r="D20" t="str">
         <v>-</v>
       </c>
-      <c r="D20" t="str">
+      <c r="E20" t="str">
         <v>Increase ELEMENT damage</v>
       </c>
-      <c r="E20" t="str">
+      <c r="F20" t="str">
         <v>Increase ELEMENT damage received by X%</v>
       </c>
-      <c r="F20" t="str">
+      <c r="G20" t="str">
         <v>10</v>
       </c>
-      <c r="G20" t="str">
+      <c r="H20" t="str">
         <v>Percent</v>
       </c>
     </row>
@@ -928,21 +988,24 @@
         <v>squishy</v>
       </c>
       <c r="B21" t="str">
-        <v>Active</v>
+        <v>Fire, Earth</v>
       </c>
       <c r="C21" t="str">
+        <v>Active</v>
+      </c>
+      <c r="D21" t="str">
         <v>-</v>
       </c>
-      <c r="D21" t="str">
-        <v>Removes X% shield</v>
-      </c>
       <c r="E21" t="str">
-        <v>Removes X% of shield from attacker when used</v>
+        <v>Removes X% of your shield on use</v>
       </c>
       <c r="F21" t="str">
+        <v>Removes X% of your shield when used</v>
+      </c>
+      <c r="G21" t="str">
         <v>100</v>
       </c>
-      <c r="G21" t="str">
+      <c r="H21" t="str">
         <v>Percent</v>
       </c>
     </row>
@@ -951,21 +1014,24 @@
         <v>multihit</v>
       </c>
       <c r="B22" t="str">
-        <v>Active</v>
+        <v>Lightning</v>
       </c>
       <c r="C22" t="str">
-        <v>+</v>
+        <v>Active</v>
       </c>
       <c r="D22" t="str">
+        <v>+</v>
+      </c>
+      <c r="E22" t="str">
         <v>Hits multiple times</v>
       </c>
-      <c r="E22" t="str">
+      <c r="F22" t="str">
         <v>Triggers X times on use</v>
       </c>
-      <c r="F22" t="str">
+      <c r="G22" t="str">
         <v>2</v>
       </c>
-      <c r="G22" t="str">
+      <c r="H22" t="str">
         <v>Number</v>
       </c>
     </row>
@@ -974,21 +1040,24 @@
         <v>exhaust</v>
       </c>
       <c r="B23" t="str">
-        <v>Active</v>
+        <v>Air, Water</v>
       </c>
       <c r="C23" t="str">
+        <v>Active</v>
+      </c>
+      <c r="D23" t="str">
         <v>-</v>
       </c>
-      <c r="D23" t="str">
+      <c r="E23" t="str">
         <v>Remove X% of energy on use</v>
       </c>
-      <c r="E23" t="str">
+      <c r="F23" t="str">
         <v>Removes X% of energy when used</v>
       </c>
-      <c r="F23" t="str">
+      <c r="G23" t="str">
         <v>100</v>
       </c>
-      <c r="G23" t="str">
+      <c r="H23" t="str">
         <v>Percent</v>
       </c>
     </row>
@@ -997,21 +1066,24 @@
         <v>powerful</v>
       </c>
       <c r="B24" t="str">
+        <v>Soul</v>
+      </c>
+      <c r="C24" t="str">
         <v>Creation</v>
       </c>
-      <c r="C24" t="str">
-        <v>+</v>
-      </c>
       <c r="D24" t="str">
+        <v>+</v>
+      </c>
+      <c r="E24" t="str">
         <v>Enhances damage</v>
       </c>
-      <c r="E24" t="str">
+      <c r="F24" t="str">
         <v>Increase damage by X% on creation</v>
       </c>
-      <c r="F24" t="str">
+      <c r="G24" t="str">
         <v>250</v>
       </c>
-      <c r="G24" t="str">
+      <c r="H24" t="str">
         <v>Percent</v>
       </c>
     </row>
@@ -1020,21 +1092,24 @@
         <v>energetic</v>
       </c>
       <c r="B25" t="str">
+        <v>Soul</v>
+      </c>
+      <c r="C25" t="str">
         <v>Creation</v>
       </c>
-      <c r="C25" t="str">
-        <v>+</v>
-      </c>
       <c r="D25" t="str">
+        <v>+</v>
+      </c>
+      <c r="E25" t="str">
         <v>Decreases energy cost</v>
       </c>
-      <c r="E25" t="str">
+      <c r="F25" t="str">
         <v>Decrease energy cost by X on creation</v>
       </c>
-      <c r="F25" t="str">
+      <c r="G25" t="str">
         <v>1</v>
       </c>
-      <c r="G25" t="str">
+      <c r="H25" t="str">
         <v>Number</v>
       </c>
     </row>
@@ -1043,21 +1118,24 @@
         <v>efficient</v>
       </c>
       <c r="B26" t="str">
+        <v>Soul</v>
+      </c>
+      <c r="C26" t="str">
         <v>Creation</v>
       </c>
-      <c r="C26" t="str">
-        <v>+</v>
-      </c>
       <c r="D26" t="str">
+        <v>+</v>
+      </c>
+      <c r="E26" t="str">
         <v>Enhances effects</v>
       </c>
-      <c r="E26" t="str">
+      <c r="F26" t="str">
         <v>Increases value of effect by X% on creation</v>
       </c>
-      <c r="F26" t="str">
+      <c r="G26" t="str">
         <v>150</v>
       </c>
-      <c r="G26" t="str">
+      <c r="H26" t="str">
         <v>Percent</v>
       </c>
     </row>
@@ -1066,21 +1144,24 @@
         <v>boosted</v>
       </c>
       <c r="B27" t="str">
+        <v>Air, Lightning</v>
+      </c>
+      <c r="C27" t="str">
         <v>Passive</v>
       </c>
-      <c r="C27" t="str">
-        <v>+</v>
-      </c>
       <c r="D27" t="str">
+        <v>+</v>
+      </c>
+      <c r="E27" t="str">
         <v>Increases energy at turn start</v>
       </c>
-      <c r="E27" t="str">
+      <c r="F27" t="str">
         <v>+X energy at turn start</v>
       </c>
-      <c r="F27" t="str">
+      <c r="G27" t="str">
         <v>1</v>
       </c>
-      <c r="G27" t="str">
+      <c r="H27" t="str">
         <v>Number</v>
       </c>
     </row>
@@ -1089,21 +1170,24 @@
         <v>healthy</v>
       </c>
       <c r="B28" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="C28" t="str">
         <v>Passive</v>
       </c>
-      <c r="C28" t="str">
-        <v>+</v>
-      </c>
       <c r="D28" t="str">
+        <v>+</v>
+      </c>
+      <c r="E28" t="str">
         <v>Increases Max HP</v>
       </c>
-      <c r="E28" t="str">
+      <c r="F28" t="str">
         <v>+X Max HP</v>
       </c>
-      <c r="F28" t="str">
+      <c r="G28" t="str">
         <v>10</v>
       </c>
-      <c r="G28" t="str">
+      <c r="H28" t="str">
         <v>Number</v>
       </c>
     </row>
@@ -1112,27 +1196,160 @@
         <v>unstable</v>
       </c>
       <c r="B29" t="str">
+        <v>Soul</v>
+      </c>
+      <c r="C29" t="str">
         <v>Element</v>
       </c>
-      <c r="C29" t="str">
-        <v>+</v>
-      </c>
       <c r="D29" t="str">
-        <v>Consumed after X uses in a FORMULA</v>
+        <v>+</v>
       </c>
       <c r="E29" t="str">
         <v>Consumed after X uses in a FORMULA</v>
       </c>
       <c r="F29" t="str">
+        <v>Consumed after X uses in a FORMULA</v>
+      </c>
+      <c r="G29" t="str">
         <v>1</v>
       </c>
-      <c r="G29" t="str">
+      <c r="H29" t="str">
         <v>Number</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>gust</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Air</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Active</v>
+      </c>
+      <c r="D30" t="str">
+        <v>+</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Increase FIRE Damage on next attack</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Increases FIRE Damage by X% on next attack</v>
+      </c>
+      <c r="G30" t="str">
+        <v>50</v>
+      </c>
+      <c r="H30" t="str">
+        <v>Percent</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>root</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Active</v>
+      </c>
+      <c r="D31" t="str">
+        <v>+</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Increase WATER Damage on next attack</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Increases WATER Damage by X% on next attack</v>
+      </c>
+      <c r="G31" t="str">
+        <v>50</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Percent</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>static</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Active</v>
+      </c>
+      <c r="D32" t="str">
+        <v>+</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Increase EARTH Damage on next attack</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Increases EARTH Damage by X% on next attack</v>
+      </c>
+      <c r="G32" t="str">
+        <v>50</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Percent</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>flame</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Active</v>
+      </c>
+      <c r="D33" t="str">
+        <v>+</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Increase AIR Damage on next attack</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Increases AIR Damage by X% on next attack</v>
+      </c>
+      <c r="G33" t="str">
+        <v>50</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Percent</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>drizzle</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Water</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Active</v>
+      </c>
+      <c r="D34" t="str">
+        <v>+</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Increase LIGHTNING Damage on next attack</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Increases LIGHTNING Damage by X% on next attack</v>
+      </c>
+      <c r="G34" t="str">
+        <v>50</v>
+      </c>
+      <c r="H34" t="str">
+        <v>Percent</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J34"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>